<commit_message>
Confirm transferred work dates in base acts
</commit_message>
<xml_diff>
--- a/output/spreadsheet/Основная таблица ИБ12 (ВК).xlsx
+++ b/output/spreadsheet/Основная таблица ИБ12 (ВК).xlsx
@@ -135,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -234,6 +234,27 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -699,10 +720,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +7.650, 3 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G2" s="27" t="n">
+      <c r="G2" s="34" t="n">
         <v>45477</v>
       </c>
-      <c r="H2" s="27" t="n">
+      <c r="H2" s="34" t="n">
         <v>45479</v>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -743,10 +764,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +10.650, 4 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G3" s="27" t="n">
+      <c r="G3" s="34" t="n">
         <v>45480</v>
       </c>
-      <c r="H3" s="27" t="n">
+      <c r="H3" s="34" t="n">
         <v>45481</v>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -787,10 +808,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +13.650, 5 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G4" s="27" t="n">
+      <c r="G4" s="34" t="n">
         <v>45482</v>
       </c>
-      <c r="H4" s="27" t="n">
+      <c r="H4" s="34" t="n">
         <v>45483</v>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -831,10 +852,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +16.650, 6 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="34" t="n">
         <v>45484</v>
       </c>
-      <c r="H5" s="27" t="n">
+      <c r="H5" s="34" t="n">
         <v>45488</v>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -875,10 +896,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +19.650, 7 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="34" t="n">
         <v>45489</v>
       </c>
-      <c r="H6" s="27" t="n">
+      <c r="H6" s="34" t="n">
         <v>45492</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -919,10 +940,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +22.650, 8 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="34" t="n">
         <v>45518</v>
       </c>
-      <c r="H7" s="27" t="n">
+      <c r="H7" s="34" t="n">
         <v>45522</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -963,10 +984,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +25.650, 9 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="34" t="n">
         <v>45527</v>
       </c>
-      <c r="H8" s="27" t="n">
+      <c r="H8" s="34" t="n">
         <v>45531</v>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1007,10 +1028,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов 1 из сшитого полиэтилена систем В1.1, Т3.1 на отм. +28.650, 10 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="34" t="n">
         <v>45539</v>
       </c>
-      <c r="H9" s="27" t="n">
+      <c r="H9" s="34" t="n">
         <v>45543</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1051,10 +1072,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +31.650, 11 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G10" s="27" t="n">
+      <c r="G10" s="34" t="n">
         <v>45544</v>
       </c>
-      <c r="H10" s="27" t="n">
+      <c r="H10" s="34" t="n">
         <v>45548</v>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1095,10 +1116,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +34.650, 12 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G11" s="27" t="n">
+      <c r="G11" s="34" t="n">
         <v>45549</v>
       </c>
-      <c r="H11" s="27" t="n">
+      <c r="H11" s="34" t="n">
         <v>45553</v>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1139,10 +1160,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +37.650, 13 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="34" t="n">
         <v>45554</v>
       </c>
-      <c r="H12" s="27" t="n">
+      <c r="H12" s="34" t="n">
         <v>45587</v>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1183,10 +1204,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +40.650, 14 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G13" s="27" t="n">
+      <c r="G13" s="34" t="n">
         <v>45558</v>
       </c>
-      <c r="H13" s="27" t="n">
+      <c r="H13" s="34" t="n">
         <v>45561</v>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1227,10 +1248,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов 1 из сшитого полиэтилена систем В1.1, Т3.1 на отм. +43.650, 15 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="34" t="n">
         <v>45562</v>
       </c>
-      <c r="H14" s="27" t="n">
+      <c r="H14" s="34" t="n">
         <v>45565</v>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1271,10 +1292,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +46.650, 16 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G15" s="27" t="n">
+      <c r="G15" s="34" t="n">
         <v>45566</v>
       </c>
-      <c r="H15" s="27" t="n">
+      <c r="H15" s="34" t="n">
         <v>45569</v>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1315,10 +1336,10 @@
           <t>Монтаж полипропиленовых трубопроводов, гильз для стояков и горизонтальных трубопроводов, неподвижных опор и запорной арматуры систем В1.1,Т3.1,Т4.1 с отм. -0.780 до отм. +48.150, с подвала по 16 этаж в/о 1с-10с/Ас-Ис (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G16" s="27" t="n">
+      <c r="G16" s="34" t="n">
         <v>45570</v>
       </c>
-      <c r="H16" s="27" t="n">
+      <c r="H16" s="34" t="n">
         <v>45573</v>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1359,10 +1380,10 @@
           <t>Монтаж этажных распределительных коллекторов систем В1.1, Т3.1 с отм. +4.650 до отм +46.650, со 2 по 16 этаж в/о 9с-10с/Вс-Гс</t>
         </is>
       </c>
-      <c r="G17" s="27" t="n">
+      <c r="G17" s="34" t="n">
         <v>45673</v>
       </c>
-      <c r="H17" s="27" t="n">
+      <c r="H17" s="34" t="n">
         <v>45698</v>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1403,10 +1424,10 @@
           <t>Монтаж трубопроводов и запорной арматуры к сантехническому оборудованию систем В1.1, Т3.1 с отм. +0.140 до отм +46.650, с 1 по 16 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G18" s="27" t="n">
+      <c r="G18" s="34" t="n">
         <v>45960</v>
       </c>
-      <c r="H18" s="27" t="n">
+      <c r="H18" s="34" t="n">
         <v>45962</v>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1447,10 +1468,10 @@
           <t>Монтаж водомерных узлов сетей В1.1, Т3.1 на отм. +0.140, 1 этаж в/о 2с-6с/Бс-Дс (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G19" s="27" t="n">
+      <c r="G19" s="34" t="n">
         <v>45807</v>
       </c>
-      <c r="H19" s="27" t="n">
+      <c r="H19" s="34" t="n">
         <v>45841</v>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1491,10 +1512,10 @@
           <t>Монтаж гибких подводок и смесителей систем В1.1, Т3.1 с отм. +0.140 до отм +46.650, с 1 по 16 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G20" s="27" t="n">
+      <c r="G20" s="34" t="n">
         <v>45974</v>
       </c>
-      <c r="H20" s="27" t="n">
+      <c r="H20" s="34" t="n">
         <v>45974</v>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1535,10 +1556,10 @@
           <t>Монтаж устройства внутриквартирного пожаротушения систем В1.1 с отм. +4.650 до отм +46.650, со 2 по 16 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G21" s="27" t="n">
+      <c r="G21" s="34" t="n">
         <v>45954</v>
       </c>
-      <c r="H21" s="27" t="n">
+      <c r="H21" s="34" t="n">
         <v>45969</v>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1579,10 +1600,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов систем В1.1,Т3.1,Т4.1 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="34" t="n">
         <v>45954</v>
       </c>
-      <c r="H22" s="27" t="n">
+      <c r="H22" s="34" t="n">
         <v>45969</v>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1619,8 +1640,8 @@
         </is>
       </c>
       <c r="F23" s="7" t="n"/>
-      <c r="G23" s="28" t="n"/>
-      <c r="H23" s="28" t="n"/>
+      <c r="G23" s="35" t="n"/>
+      <c r="H23" s="35" t="n"/>
       <c r="I23" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -1659,10 +1680,10 @@
           <t>Изоляция полипропиленовых трубопроводов систем В1.1,Т3.1,Т4.1 с отм. -0.780 до отм. +48.150, с подвала по 16 этаж в/о 2с-11с/Ас-Ис (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G24" s="27" t="n">
+      <c r="G24" s="34" t="n">
         <v>45699</v>
       </c>
-      <c r="H24" s="27" t="n">
+      <c r="H24" s="34" t="n">
         <v>45702</v>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1703,10 +1724,10 @@
           <t>Проведение промывки трубопроводов системы ХВС (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G25" s="27" t="n">
+      <c r="G25" s="34" t="n">
         <v>45703</v>
       </c>
-      <c r="H25" s="27" t="n">
+      <c r="H25" s="34" t="n">
         <v>45707</v>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1743,8 +1764,8 @@
         </is>
       </c>
       <c r="F26" s="9" t="n"/>
-      <c r="G26" s="29" t="n"/>
-      <c r="H26" s="29" t="n"/>
+      <c r="G26" s="36" t="n"/>
+      <c r="H26" s="36" t="n"/>
       <c r="I26" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -1779,8 +1800,8 @@
         </is>
       </c>
       <c r="F27" s="9" t="n"/>
-      <c r="G27" s="29" t="n"/>
-      <c r="H27" s="29" t="n"/>
+      <c r="G27" s="36" t="n"/>
+      <c r="H27" s="36" t="n"/>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -1815,8 +1836,8 @@
         </is>
       </c>
       <c r="F28" s="9" t="n"/>
-      <c r="G28" s="29" t="n"/>
-      <c r="H28" s="29" t="n"/>
+      <c r="G28" s="36" t="n"/>
+      <c r="H28" s="36" t="n"/>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -1851,8 +1872,8 @@
         </is>
       </c>
       <c r="F29" s="9" t="n"/>
-      <c r="G29" s="29" t="n"/>
-      <c r="H29" s="29" t="n"/>
+      <c r="G29" s="36" t="n"/>
+      <c r="H29" s="36" t="n"/>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -1887,8 +1908,8 @@
         </is>
       </c>
       <c r="F30" s="9" t="n"/>
-      <c r="G30" s="29" t="n"/>
-      <c r="H30" s="29" t="n"/>
+      <c r="G30" s="36" t="n"/>
+      <c r="H30" s="36" t="n"/>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -1931,10 +1952,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +52.650, 18 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G31" s="27" t="n">
+      <c r="G31" s="34" t="n">
         <v>45576</v>
       </c>
-      <c r="H31" s="27" t="n">
+      <c r="H31" s="34" t="n">
         <v>45578</v>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -1975,10 +1996,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +55.650, 19 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G32" s="27" t="n">
+      <c r="G32" s="34" t="n">
         <v>45579</v>
       </c>
-      <c r="H32" s="27" t="n">
+      <c r="H32" s="34" t="n">
         <v>45580</v>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2019,10 +2040,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +58.650, 20 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G33" s="27" t="n">
+      <c r="G33" s="34" t="n">
         <v>45581</v>
       </c>
-      <c r="H33" s="27" t="n">
+      <c r="H33" s="34" t="n">
         <v>45582</v>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -2063,10 +2084,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +61.650, 21 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G34" s="27" t="n">
+      <c r="G34" s="34" t="n">
         <v>45583</v>
       </c>
-      <c r="H34" s="27" t="n">
+      <c r="H34" s="34" t="n">
         <v>45585</v>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2107,10 +2128,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +64.650, 22 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G35" s="27" t="n">
+      <c r="G35" s="34" t="n">
         <v>45586</v>
       </c>
-      <c r="H35" s="27" t="n">
+      <c r="H35" s="34" t="n">
         <v>45587</v>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -2151,10 +2172,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +67.650, 23 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G36" s="27" t="n">
+      <c r="G36" s="34" t="n">
         <v>45588</v>
       </c>
-      <c r="H36" s="27" t="n">
+      <c r="H36" s="34" t="n">
         <v>45590</v>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -2195,10 +2216,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +70.650, 24 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G37" s="27" t="n">
+      <c r="G37" s="34" t="n">
         <v>45634</v>
       </c>
-      <c r="H37" s="27" t="n">
+      <c r="H37" s="34" t="n">
         <v>45635</v>
       </c>
       <c r="I37" s="4" t="inlineStr">
@@ -2239,10 +2260,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +73.650, 25 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G38" s="27" t="n">
+      <c r="G38" s="34" t="n">
         <v>45635</v>
       </c>
-      <c r="H38" s="27" t="n">
+      <c r="H38" s="34" t="n">
         <v>45636</v>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -2283,10 +2304,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +76.650, 26 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G39" s="27" t="n">
+      <c r="G39" s="34" t="n">
         <v>45637</v>
       </c>
-      <c r="H39" s="27" t="n">
+      <c r="H39" s="34" t="n">
         <v>45639</v>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -2327,10 +2348,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +79.650, 27 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G40" s="27" t="n">
+      <c r="G40" s="34" t="n">
         <v>45639</v>
       </c>
-      <c r="H40" s="27" t="n">
+      <c r="H40" s="34" t="n">
         <v>45641</v>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2371,10 +2392,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +82.650, 28 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G41" s="27" t="n">
+      <c r="G41" s="34" t="n">
         <v>45642</v>
       </c>
-      <c r="H41" s="27" t="n">
+      <c r="H41" s="34" t="n">
         <v>45644</v>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2415,10 +2436,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +85.650, 29 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G42" s="27" t="n">
+      <c r="G42" s="34" t="n">
         <v>45645</v>
       </c>
-      <c r="H42" s="27" t="n">
+      <c r="H42" s="34" t="n">
         <v>45648</v>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -2459,10 +2480,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +88.650, 30 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G43" s="27" t="n">
+      <c r="G43" s="34" t="n">
         <v>45649</v>
       </c>
-      <c r="H43" s="27" t="n">
+      <c r="H43" s="34" t="n">
         <v>45652</v>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -2503,10 +2524,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2на отм. +91.650, 31 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G44" s="27" t="n">
+      <c r="G44" s="34" t="n">
         <v>45684</v>
       </c>
-      <c r="H44" s="27" t="n">
+      <c r="H44" s="34" t="n">
         <v>45686</v>
       </c>
       <c r="I44" s="4" t="inlineStr">
@@ -2547,10 +2568,10 @@
           <t>Монтаж полипропиленовых трубопроводов, гильз для стояков и горизонтальных трубопроводов, неподвижных опор и запорной арматуры систем В1.2,Т3.2,Т4.2 с отм. -0.780 до отм. +93.150, с подвала по 31 этаж в/о 9с-11с/Вс-Дс (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G45" s="27" t="n">
+      <c r="G45" s="34" t="n">
         <v>45687</v>
       </c>
-      <c r="H45" s="27" t="n">
+      <c r="H45" s="34" t="n">
         <v>45689</v>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -2591,10 +2612,10 @@
           <t>Монтаж этажных распределительных коллекторов систем В1.2, Т3.2 с отм. +49.650 до отм +91.650, с 17 по 31 этаж в/о 9с-10с/Вс-Гс(Секция №12.1)</t>
         </is>
       </c>
-      <c r="G46" s="27" t="n">
+      <c r="G46" s="34" t="n">
         <v>45673</v>
       </c>
-      <c r="H46" s="27" t="n">
+      <c r="H46" s="34" t="n">
         <v>45952</v>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -2635,10 +2656,10 @@
           <t>Монтаж трубопроводов и запорной арматуры к сантехническому оборудованию систем В1.2, Т3.2 с отм. +49.650 до отм +91.650, с 17 по 31 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G47" s="27" t="n">
+      <c r="G47" s="34" t="n">
         <v>45963</v>
       </c>
-      <c r="H47" s="27" t="n">
+      <c r="H47" s="34" t="n">
         <v>45965</v>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -2679,10 +2700,10 @@
           <t>Монтаж гибких подводок и смесителей систем В1.2, Т3.2 с отм. +49.650 до отм +91.650, с 17 по 31 этаж в/о 1с-11с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G48" s="27" t="n">
+      <c r="G48" s="34" t="n">
         <v>45842</v>
       </c>
-      <c r="H48" s="27" t="n">
+      <c r="H48" s="34" t="n">
         <v>45901</v>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -2723,10 +2744,10 @@
           <t>Монтаж устройства внутриквартирного пожаротушения систем В1.2 с отм. +49.650 до отм +91.650, с 17 по 31 этаж в/о 1с-11с/Бс-Ес ( (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G49" s="27" t="n">
+      <c r="G49" s="34" t="n">
         <v>45970</v>
       </c>
-      <c r="H49" s="27" t="n">
+      <c r="H49" s="34" t="n">
         <v>45982</v>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -2767,10 +2788,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов систем В1.2,Т3.2,Т4.2 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G50" s="27" t="n">
+      <c r="G50" s="34" t="n">
         <v>45970</v>
       </c>
-      <c r="H50" s="27" t="n">
+      <c r="H50" s="34" t="n">
         <v>45982</v>
       </c>
       <c r="I50" s="4" t="inlineStr">
@@ -2807,8 +2828,8 @@
         </is>
       </c>
       <c r="F51" s="7" t="n"/>
-      <c r="G51" s="28" t="n"/>
-      <c r="H51" s="28" t="n"/>
+      <c r="G51" s="35" t="n"/>
+      <c r="H51" s="35" t="n"/>
       <c r="I51" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -2847,10 +2868,10 @@
           <t>Изоляция полипропиленовых трубопроводов с отм. -0.780 до отм. +93.150, с подвала по 31 этаж в/о 9с-11с/Вс-Дс систем В1.2,Т3.2,Т4.2 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G52" s="27" t="n">
+      <c r="G52" s="34" t="n">
         <v>45953</v>
       </c>
-      <c r="H52" s="27" t="n">
+      <c r="H52" s="34" t="n">
         <v>45956</v>
       </c>
       <c r="I52" s="4" t="inlineStr">
@@ -2891,10 +2912,10 @@
           <t>Проведение промывки трубопроводов системы ХВС (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G53" s="27" t="n">
+      <c r="G53" s="34" t="n">
         <v>45957</v>
       </c>
-      <c r="H53" s="27" t="n">
+      <c r="H53" s="34" t="n">
         <v>45961</v>
       </c>
       <c r="I53" s="4" t="inlineStr">
@@ -2931,8 +2952,8 @@
         </is>
       </c>
       <c r="F54" s="9" t="n"/>
-      <c r="G54" s="29" t="n"/>
-      <c r="H54" s="29" t="n"/>
+      <c r="G54" s="36" t="n"/>
+      <c r="H54" s="36" t="n"/>
       <c r="I54" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -2967,8 +2988,8 @@
         </is>
       </c>
       <c r="F55" s="9" t="n"/>
-      <c r="G55" s="29" t="n"/>
-      <c r="H55" s="29" t="n"/>
+      <c r="G55" s="36" t="n"/>
+      <c r="H55" s="36" t="n"/>
       <c r="I55" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3003,8 +3024,8 @@
         </is>
       </c>
       <c r="F56" s="9" t="n"/>
-      <c r="G56" s="29" t="n"/>
-      <c r="H56" s="29" t="n"/>
+      <c r="G56" s="36" t="n"/>
+      <c r="H56" s="36" t="n"/>
       <c r="I56" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3039,8 +3060,8 @@
         </is>
       </c>
       <c r="F57" s="9" t="n"/>
-      <c r="G57" s="29" t="n"/>
-      <c r="H57" s="29" t="n"/>
+      <c r="G57" s="36" t="n"/>
+      <c r="H57" s="36" t="n"/>
       <c r="I57" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3075,8 +3096,8 @@
         </is>
       </c>
       <c r="F58" s="9" t="n"/>
-      <c r="G58" s="29" t="n"/>
-      <c r="H58" s="29" t="n"/>
+      <c r="G58" s="36" t="n"/>
+      <c r="H58" s="36" t="n"/>
       <c r="I58" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3120,10 +3141,10 @@
           <t>Монтаж трубопроводов к сантехническому оборудованию системы бытовой канализации К1 с отм. +4.650 до отм. +91.650, со 2 по 31 этаж в/о 1с-11с/Ас-Ис (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G59" s="27" t="n">
+      <c r="G59" s="34" t="n">
         <v>45513</v>
       </c>
-      <c r="H59" s="27" t="n">
+      <c r="H59" s="34" t="n">
         <v>45748</v>
       </c>
       <c r="I59" s="4" t="inlineStr">
@@ -3164,10 +3185,10 @@
           <t>Монтаж сантехнического оборудования системы бытовой канализации К1 с отм. +4.650 до отм. +91.650, со 2 по 31 этаж в/о 1с-11с/Ас-Ис (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G60" s="27" t="n">
+      <c r="G60" s="34" t="n">
         <v>45847</v>
       </c>
-      <c r="H60" s="27" t="n">
+      <c r="H60" s="34" t="n">
         <v>45910</v>
       </c>
       <c r="I60" s="4" t="inlineStr">
@@ -3208,10 +3229,10 @@
           <t>Проведение испытания систем канализации и водостоков системы бытовой канализации К1 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G61" s="27" t="n">
+      <c r="G61" s="34" t="n">
         <v>45954</v>
       </c>
-      <c r="H61" s="27" t="n">
+      <c r="H61" s="34" t="n">
         <v>45969</v>
       </c>
       <c r="I61" s="4" t="inlineStr">
@@ -3248,8 +3269,8 @@
         </is>
       </c>
       <c r="F62" s="11" t="n"/>
-      <c r="G62" s="30" t="n"/>
-      <c r="H62" s="30" t="n"/>
+      <c r="G62" s="37" t="n"/>
+      <c r="H62" s="37" t="n"/>
       <c r="I62" s="10" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3284,8 +3305,8 @@
         </is>
       </c>
       <c r="F63" s="9" t="n"/>
-      <c r="G63" s="29" t="n"/>
-      <c r="H63" s="29" t="n"/>
+      <c r="G63" s="36" t="n"/>
+      <c r="H63" s="36" t="n"/>
       <c r="I63" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3328,10 +3349,10 @@
           <t>Монтаж трубопроводов к сантехническому оборудованию системы бытовой канализации встроенных помещений К1.1 на отм. +0.140, 1 этаж в/о 2с-8с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G64" s="27" t="n">
+      <c r="G64" s="34" t="n">
         <v>45982</v>
       </c>
-      <c r="H64" s="27" t="n">
+      <c r="H64" s="34" t="n">
         <v>45983</v>
       </c>
       <c r="I64" s="4" t="inlineStr">
@@ -3376,10 +3397,10 @@
           <t>Монтаж сантехнического оборудования системы бытовой канализации встроенных помещений К1.1 на отм. +0.140, 1 этаж в/о 2с-8с/Бс-Ес (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G65" s="27" t="n">
+      <c r="G65" s="34" t="n">
         <v>45984</v>
       </c>
-      <c r="H65" s="27" t="n">
+      <c r="H65" s="34" t="n">
         <v>45984</v>
       </c>
       <c r="I65" s="4" t="inlineStr">
@@ -3424,10 +3445,10 @@
           <t>Проведение испытания систем канализации и водостоков системы бытовой канализации встроенных помещений К1.1 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G66" s="27" t="n">
+      <c r="G66" s="34" t="n">
         <v>45985</v>
       </c>
-      <c r="H66" s="27" t="n">
+      <c r="H66" s="34" t="n">
         <v>45985</v>
       </c>
       <c r="I66" s="4" t="inlineStr">
@@ -3468,8 +3489,8 @@
         </is>
       </c>
       <c r="F67" s="11" t="n"/>
-      <c r="G67" s="30" t="n"/>
-      <c r="H67" s="30" t="n"/>
+      <c r="G67" s="37" t="n"/>
+      <c r="H67" s="37" t="n"/>
       <c r="I67" s="10" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3504,8 +3525,8 @@
         </is>
       </c>
       <c r="F68" s="9" t="n"/>
-      <c r="G68" s="29" t="n"/>
-      <c r="H68" s="29" t="n"/>
+      <c r="G68" s="36" t="n"/>
+      <c r="H68" s="36" t="n"/>
       <c r="I68" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3549,10 +3570,10 @@
           <t>Проведение испытания систем канализации и водостоков системы внутреннего водостока К2 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G69" s="27" t="n">
+      <c r="G69" s="34" t="n">
         <v>45520</v>
       </c>
-      <c r="H69" s="27" t="n">
+      <c r="H69" s="34" t="n">
         <v>45953</v>
       </c>
       <c r="I69" s="4" t="inlineStr">
@@ -3594,8 +3615,8 @@
         </is>
       </c>
       <c r="F70" s="11" t="n"/>
-      <c r="G70" s="30" t="n"/>
-      <c r="H70" s="30" t="n"/>
+      <c r="G70" s="37" t="n"/>
+      <c r="H70" s="37" t="n"/>
       <c r="I70" s="10" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3634,10 +3655,10 @@
           <t>Освидетельствование участков сетей инженерно-технического обеспечения системы внутреннего водостока К2 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G71" s="27" t="n">
+      <c r="G71" s="34" t="n">
         <v>45954</v>
       </c>
-      <c r="H71" s="27" t="n">
+      <c r="H71" s="34" t="n">
         <v>45956</v>
       </c>
       <c r="I71" s="4" t="inlineStr">
@@ -3674,8 +3695,8 @@
         </is>
       </c>
       <c r="F72" s="9" t="n"/>
-      <c r="G72" s="29" t="n"/>
-      <c r="H72" s="29" t="n"/>
+      <c r="G72" s="36" t="n"/>
+      <c r="H72" s="36" t="n"/>
       <c r="I72" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3718,10 +3739,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов системы напорной дренажной канализации К13, К13н (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G73" s="27" t="n">
+      <c r="G73" s="34" t="n">
         <v>45523</v>
       </c>
-      <c r="H73" s="27" t="n">
+      <c r="H73" s="34" t="n">
         <v>45953</v>
       </c>
       <c r="I73" s="4" t="inlineStr">
@@ -3758,8 +3779,8 @@
         </is>
       </c>
       <c r="F74" s="7" t="n"/>
-      <c r="G74" s="28" t="n"/>
-      <c r="H74" s="28" t="n"/>
+      <c r="G74" s="35" t="n"/>
+      <c r="H74" s="35" t="n"/>
       <c r="I74" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -3798,10 +3819,10 @@
           <t>Проведение испытания систем канализации и водостоков системы напорной дренажной канализации К13, К13н (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G75" s="27" t="n">
+      <c r="G75" s="34" t="n">
         <v>45954</v>
       </c>
-      <c r="H75" s="27" t="n">
+      <c r="H75" s="34" t="n">
         <v>45954</v>
       </c>
       <c r="I75" s="4" t="inlineStr">
@@ -3838,8 +3859,8 @@
         </is>
       </c>
       <c r="F76" s="11" t="n"/>
-      <c r="G76" s="30" t="n"/>
-      <c r="H76" s="30" t="n"/>
+      <c r="G76" s="37" t="n"/>
+      <c r="H76" s="37" t="n"/>
       <c r="I76" s="10" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3874,8 +3895,8 @@
         </is>
       </c>
       <c r="F77" s="13" t="n"/>
-      <c r="G77" s="31" t="n"/>
-      <c r="H77" s="31" t="n"/>
+      <c r="G77" s="38" t="n"/>
+      <c r="H77" s="38" t="n"/>
       <c r="I77" s="12" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3910,8 +3931,8 @@
         </is>
       </c>
       <c r="F78" s="9" t="n"/>
-      <c r="G78" s="29" t="n"/>
-      <c r="H78" s="29" t="n"/>
+      <c r="G78" s="36" t="n"/>
+      <c r="H78" s="36" t="n"/>
       <c r="I78" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -3954,10 +3975,10 @@
           <t>Монтаж пожарного оборудования системы противопожарного водопровода В2.1 с отм. -3.350 до отм. +49.150, с подвала по 16 этаж в/о 1с-11с/Ас-Жс (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G79" s="27" t="n">
+      <c r="G79" s="34" t="n">
         <v>45478</v>
       </c>
-      <c r="H79" s="27" t="n">
+      <c r="H79" s="34" t="n">
         <v>45917</v>
       </c>
       <c r="I79" s="4" t="inlineStr">
@@ -3998,10 +4019,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов системы противопожарного водопровода В2.1 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G80" s="27" t="n">
+      <c r="G80" s="34" t="n">
         <v>45478</v>
       </c>
-      <c r="H80" s="27" t="n">
+      <c r="H80" s="34" t="n">
         <v>45917</v>
       </c>
       <c r="I80" s="4" t="inlineStr">
@@ -4038,8 +4059,8 @@
         </is>
       </c>
       <c r="F81" s="7" t="n"/>
-      <c r="G81" s="28" t="n"/>
-      <c r="H81" s="28" t="n"/>
+      <c r="G81" s="35" t="n"/>
+      <c r="H81" s="35" t="n"/>
       <c r="I81" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -4078,10 +4099,10 @@
           <t>Зачеканка гильз в местах прохода через ограждающие конструкции трубопроводов системы противопожарного водопровода В2.1 с отм. -0.970 до отм. +46.650, с подвала по 16 этаж в/о 1с-11с/Ас-Жс (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G82" s="27" t="n">
+      <c r="G82" s="34" t="n">
         <v>45918</v>
       </c>
-      <c r="H82" s="27" t="n">
+      <c r="H82" s="34" t="n">
         <v>45919</v>
       </c>
       <c r="I82" s="4" t="inlineStr">
@@ -4127,10 +4148,10 @@
           <t>Испытание на водоотдачу внутреннего противопожарного водопровода (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G83" s="27" t="n">
+      <c r="G83" s="34" t="n">
         <v>45920</v>
       </c>
-      <c r="H83" s="27" t="n">
+      <c r="H83" s="34" t="n">
         <v>45921</v>
       </c>
       <c r="I83" s="4" t="inlineStr">
@@ -4167,8 +4188,8 @@
         </is>
       </c>
       <c r="F84" s="9" t="n"/>
-      <c r="G84" s="29" t="n"/>
-      <c r="H84" s="29" t="n"/>
+      <c r="G84" s="36" t="n"/>
+      <c r="H84" s="36" t="n"/>
       <c r="I84" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4203,8 +4224,8 @@
         </is>
       </c>
       <c r="F85" s="15" t="n"/>
-      <c r="G85" s="32" t="n"/>
-      <c r="H85" s="32" t="n"/>
+      <c r="G85" s="39" t="n"/>
+      <c r="H85" s="39" t="n"/>
       <c r="I85" s="14" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4239,8 +4260,8 @@
         </is>
       </c>
       <c r="F86" s="9" t="n"/>
-      <c r="G86" s="29" t="n"/>
-      <c r="H86" s="29" t="n"/>
+      <c r="G86" s="36" t="n"/>
+      <c r="H86" s="36" t="n"/>
       <c r="I86" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4283,10 +4304,10 @@
           <t>Монтаж пожарного оборудования системы противопожарного водопровода В2.2 с отм. +49.650 до отм. +94.930, с 17 этажа по тех. чердак в/о 3с-10с/Ас-Дс (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G87" s="27" t="n">
+      <c r="G87" s="34" t="n">
         <v>45478</v>
       </c>
-      <c r="H87" s="27" t="n">
+      <c r="H87" s="34" t="n">
         <v>45876</v>
       </c>
       <c r="I87" s="4" t="inlineStr">
@@ -4327,10 +4348,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов системы противопожарного водопровода В2.2 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G88" s="27" t="n">
+      <c r="G88" s="34" t="n">
         <v>45478</v>
       </c>
-      <c r="H88" s="27" t="n">
+      <c r="H88" s="34" t="n">
         <v>45876</v>
       </c>
       <c r="I88" s="4" t="inlineStr">
@@ -4367,8 +4388,8 @@
         </is>
       </c>
       <c r="F89" s="7" t="n"/>
-      <c r="G89" s="28" t="n"/>
-      <c r="H89" s="28" t="n"/>
+      <c r="G89" s="35" t="n"/>
+      <c r="H89" s="35" t="n"/>
       <c r="I89" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -4407,10 +4428,10 @@
           <t>Зачеканка гильз в местах прохода через ограждающие конструкции трубопроводов систем противопожарного водопровода В2.2 с отм. -0.890 до отм. +96.978, с подвала по тех. чердак в/о 3с-10с/Бс-Дс (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G90" s="27" t="n">
+      <c r="G90" s="34" t="n">
         <v>45877</v>
       </c>
-      <c r="H90" s="27" t="n">
+      <c r="H90" s="34" t="n">
         <v>45878</v>
       </c>
       <c r="I90" s="4" t="inlineStr">
@@ -4456,10 +4477,10 @@
           <t>Испытание на водоотдачу внутреннего противопожарного водопровода (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G91" s="27" t="n">
+      <c r="G91" s="34" t="n">
         <v>45879</v>
       </c>
-      <c r="H91" s="27" t="n">
+      <c r="H91" s="34" t="n">
         <v>45880</v>
       </c>
       <c r="I91" s="4" t="inlineStr">
@@ -4496,8 +4517,8 @@
         </is>
       </c>
       <c r="F92" s="9" t="n"/>
-      <c r="G92" s="29" t="n"/>
-      <c r="H92" s="29" t="n"/>
+      <c r="G92" s="36" t="n"/>
+      <c r="H92" s="36" t="n"/>
       <c r="I92" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4532,8 +4553,8 @@
         </is>
       </c>
       <c r="F93" s="15" t="n"/>
-      <c r="G93" s="32" t="n"/>
-      <c r="H93" s="32" t="n"/>
+      <c r="G93" s="39" t="n"/>
+      <c r="H93" s="39" t="n"/>
       <c r="I93" s="14" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4568,8 +4589,8 @@
         </is>
       </c>
       <c r="F94" s="9" t="n"/>
-      <c r="G94" s="29" t="n"/>
-      <c r="H94" s="29" t="n"/>
+      <c r="G94" s="36" t="n"/>
+      <c r="H94" s="36" t="n"/>
       <c r="I94" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4612,10 +4633,10 @@
           <t>Монтаж пожарного оборудования системы автоматического пожаротушения кладовых В2 с отм. -0.548 до отм. -0.289, подвал в/о 1с-11с/Ас-Ис (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G95" s="27" t="n">
+      <c r="G95" s="34" t="n">
         <v>45982</v>
       </c>
-      <c r="H95" s="27" t="n">
+      <c r="H95" s="34" t="n">
         <v>45984</v>
       </c>
       <c r="I95" s="4" t="inlineStr">
@@ -4656,10 +4677,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов системы автоматического пожаротушения кладовых В2 (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G96" s="27" t="n">
+      <c r="G96" s="34" t="n">
         <v>45988</v>
       </c>
-      <c r="H96" s="27" t="n">
+      <c r="H96" s="34" t="n">
         <v>45988</v>
       </c>
       <c r="I96" s="4" t="inlineStr">
@@ -4696,8 +4717,8 @@
         </is>
       </c>
       <c r="F97" s="7" t="n"/>
-      <c r="G97" s="28" t="n"/>
-      <c r="H97" s="28" t="n"/>
+      <c r="G97" s="35" t="n"/>
+      <c r="H97" s="35" t="n"/>
       <c r="I97" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -4736,10 +4757,10 @@
           <t>Зачеканка гильз в местах прохода трубопроводов через ограждающие конструкции системы автоматического пожаротушения кладовых В2 с отм. -0.862 до отм. -0.422, подвал в/о 1с-11с/Ас-Ис (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G98" s="27" t="n">
+      <c r="G98" s="34" t="n">
         <v>45996</v>
       </c>
-      <c r="H98" s="27" t="n">
+      <c r="H98" s="34" t="n">
         <v>45996</v>
       </c>
       <c r="I98" s="4" t="inlineStr">
@@ -4784,10 +4805,10 @@
           <t>Испытание на водоотдачу внутреннего противопожарного водопровода (Секция №12.1)</t>
         </is>
       </c>
-      <c r="G99" s="27" t="n">
+      <c r="G99" s="34" t="n">
         <v>45999</v>
       </c>
-      <c r="H99" s="27" t="n">
+      <c r="H99" s="34" t="n">
         <v>45999</v>
       </c>
       <c r="I99" s="4" t="inlineStr">
@@ -4824,8 +4845,8 @@
         </is>
       </c>
       <c r="F100" s="9" t="n"/>
-      <c r="G100" s="29" t="n"/>
-      <c r="H100" s="29" t="n"/>
+      <c r="G100" s="36" t="n"/>
+      <c r="H100" s="36" t="n"/>
       <c r="I100" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4860,8 +4881,8 @@
         </is>
       </c>
       <c r="F101" s="17" t="n"/>
-      <c r="G101" s="33" t="n"/>
-      <c r="H101" s="33" t="n"/>
+      <c r="G101" s="40" t="n"/>
+      <c r="H101" s="40" t="n"/>
       <c r="I101" s="16" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4900,8 +4921,8 @@
         </is>
       </c>
       <c r="F102" s="15" t="n"/>
-      <c r="G102" s="32" t="n"/>
-      <c r="H102" s="32" t="n"/>
+      <c r="G102" s="39" t="n"/>
+      <c r="H102" s="39" t="n"/>
       <c r="I102" s="14" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4936,8 +4957,8 @@
         </is>
       </c>
       <c r="F103" s="9" t="n"/>
-      <c r="G103" s="29" t="n"/>
-      <c r="H103" s="29" t="n"/>
+      <c r="G103" s="36" t="n"/>
+      <c r="H103" s="36" t="n"/>
       <c r="I103" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -4980,10 +5001,10 @@
           <t>Монтаж основного водомерного узла системы В1 с отм. -2.580 до отм. -2.253, подвал в/о 1с-2с/Ес-Жс (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G104" s="27" t="n">
+      <c r="G104" s="34" t="n">
         <v>45964</v>
       </c>
-      <c r="H104" s="27" t="n">
+      <c r="H104" s="34" t="n">
         <v>45964</v>
       </c>
       <c r="I104" s="4" t="inlineStr">
@@ -5024,10 +5045,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +4.650, 2 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G105" s="27" t="n">
+      <c r="G105" s="34" t="n">
         <v>45964</v>
       </c>
-      <c r="H105" s="27" t="n">
+      <c r="H105" s="34" t="n">
         <v>45964</v>
       </c>
       <c r="I105" s="4" t="inlineStr">
@@ -5068,10 +5089,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +7.650, 3 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G106" s="27" t="n">
+      <c r="G106" s="34" t="n">
         <v>45524</v>
       </c>
-      <c r="H106" s="27" t="n">
+      <c r="H106" s="34" t="n">
         <v>45527</v>
       </c>
       <c r="I106" s="4" t="inlineStr">
@@ -5116,10 +5137,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +10.650, 4 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G107" s="27" t="n">
+      <c r="G107" s="34" t="n">
         <v>45524</v>
       </c>
-      <c r="H107" s="27" t="n">
+      <c r="H107" s="34" t="n">
         <v>45527</v>
       </c>
       <c r="I107" s="4" t="inlineStr">
@@ -5160,10 +5181,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +13.650, 5 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G108" s="27" t="n">
+      <c r="G108" s="34" t="n">
         <v>45538</v>
       </c>
-      <c r="H108" s="27" t="n">
+      <c r="H108" s="34" t="n">
         <v>45541</v>
       </c>
       <c r="I108" s="4" t="inlineStr">
@@ -5204,10 +5225,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +16.650, 6 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G109" s="27" t="n">
+      <c r="G109" s="34" t="n">
         <v>45542</v>
       </c>
-      <c r="H109" s="27" t="n">
+      <c r="H109" s="34" t="n">
         <v>45545</v>
       </c>
       <c r="I109" s="4" t="inlineStr">
@@ -5248,10 +5269,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +19.650, 7 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G110" s="27" t="n">
+      <c r="G110" s="34" t="n">
         <v>45546</v>
       </c>
-      <c r="H110" s="27" t="n">
+      <c r="H110" s="34" t="n">
         <v>45549</v>
       </c>
       <c r="I110" s="4" t="inlineStr">
@@ -5292,10 +5313,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +22.650, 8 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G111" s="27" t="n">
+      <c r="G111" s="34" t="n">
         <v>45550</v>
       </c>
-      <c r="H111" s="27" t="n">
+      <c r="H111" s="34" t="n">
         <v>45553</v>
       </c>
       <c r="I111" s="4" t="inlineStr">
@@ -5336,10 +5357,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +25.650, 9 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G112" s="27" t="n">
+      <c r="G112" s="34" t="n">
         <v>45554</v>
       </c>
-      <c r="H112" s="27" t="n">
+      <c r="H112" s="34" t="n">
         <v>45557</v>
       </c>
       <c r="I112" s="4" t="inlineStr">
@@ -5380,10 +5401,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов 1 из сшитого полиэтилена систем В1.1, Т3.1 на отм. +28.650, 10 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G113" s="27" t="n">
+      <c r="G113" s="34" t="n">
         <v>45567</v>
       </c>
-      <c r="H113" s="27" t="n">
+      <c r="H113" s="34" t="n">
         <v>45570</v>
       </c>
       <c r="I113" s="4" t="inlineStr">
@@ -5424,10 +5445,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +31.650, 11 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G114" s="27" t="n">
+      <c r="G114" s="34" t="n">
         <v>45571</v>
       </c>
-      <c r="H114" s="27" t="n">
+      <c r="H114" s="34" t="n">
         <v>45574</v>
       </c>
       <c r="I114" s="4" t="inlineStr">
@@ -5468,10 +5489,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +34.650, 12 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G115" s="27" t="n">
+      <c r="G115" s="34" t="n">
         <v>45575</v>
       </c>
-      <c r="H115" s="27" t="n">
+      <c r="H115" s="34" t="n">
         <v>45577</v>
       </c>
       <c r="I115" s="4" t="inlineStr">
@@ -5512,10 +5533,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +37.650, 13 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G116" s="27" t="n">
+      <c r="G116" s="34" t="n">
         <v>45578</v>
       </c>
-      <c r="H116" s="27" t="n">
+      <c r="H116" s="34" t="n">
         <v>45580</v>
       </c>
       <c r="I116" s="4" t="inlineStr">
@@ -5556,10 +5577,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +40.650, 14 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G117" s="27" t="n">
+      <c r="G117" s="34" t="n">
         <v>45603</v>
       </c>
-      <c r="H117" s="27" t="n">
+      <c r="H117" s="34" t="n">
         <v>45606</v>
       </c>
       <c r="I117" s="4" t="inlineStr">
@@ -5600,10 +5621,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +43.650, 15 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G118" s="27" t="n">
+      <c r="G118" s="34" t="n">
         <v>45607</v>
       </c>
-      <c r="H118" s="27" t="n">
+      <c r="H118" s="34" t="n">
         <v>45610</v>
       </c>
       <c r="I118" s="4" t="inlineStr">
@@ -5644,10 +5665,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.1, Т3.1 на отм. +46.650, 16 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G119" s="27" t="n">
+      <c r="G119" s="34" t="n">
         <v>45611</v>
       </c>
-      <c r="H119" s="27" t="n">
+      <c r="H119" s="34" t="n">
         <v>45614</v>
       </c>
       <c r="I119" s="4" t="inlineStr">
@@ -5688,10 +5709,10 @@
           <t>Монтаж гильз для стояков, полипропиленовых и стальных трубопроводов, неподвижных опор и запорной арматуры систем В1.1,Т3.1,Т4.1 и В1 от узла ввода до насосной с отм. -1.250 до отм. +48.150, с подвала по 16 этаж в/о 1с-10с/Ас-Ис (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G120" s="27" t="n">
+      <c r="G120" s="34" t="n">
         <v>45634</v>
       </c>
-      <c r="H120" s="27" t="n">
+      <c r="H120" s="34" t="n">
         <v>45637</v>
       </c>
       <c r="I120" s="4" t="inlineStr">
@@ -5732,10 +5753,10 @@
           <t>Монтаж этажных распределительных коллекторов систем В1.1, Т3.1 с отм. +4.650 до отм +46.650, со 2 по 16 этаж в/о 8с-9с/Вс-Гс (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G121" s="27" t="n">
+      <c r="G121" s="34" t="n">
         <v>45677</v>
       </c>
-      <c r="H121" s="27" t="n">
+      <c r="H121" s="34" t="n">
         <v>45865</v>
       </c>
       <c r="I121" s="4" t="inlineStr">
@@ -5776,10 +5797,10 @@
           <t>Монтаж трубопроводов и запорной арматуры к сантехническому оборудованию систем В1.1, Т3.1 с отм. -0.210 до отм +46.650, с 1 по 16 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G122" s="27" t="n">
+      <c r="G122" s="34" t="n">
         <v>45979</v>
       </c>
-      <c r="H122" s="27" t="n">
+      <c r="H122" s="34" t="n">
         <v>45980</v>
       </c>
       <c r="I122" s="4" t="inlineStr">
@@ -5820,10 +5841,10 @@
           <t>Монтаж водомерных узлов сетей В1.1, Т3.1 на отм. -0.210, 1 этаж в/о 8с-9с/Вс-Гс (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G123" s="27" t="n">
+      <c r="G123" s="34" t="n">
         <v>45812</v>
       </c>
-      <c r="H123" s="27" t="n">
+      <c r="H123" s="34" t="n">
         <v>45851</v>
       </c>
       <c r="I123" s="4" t="inlineStr">
@@ -5864,10 +5885,10 @@
           <t>Монтаж гибких подводок и смесителей систем В1.1, Т3.1 с отм. -0.210 до отм +46.650, с 1 по 16 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G124" s="27" t="n">
+      <c r="G124" s="34" t="n">
         <v>45974</v>
       </c>
-      <c r="H124" s="27" t="n">
+      <c r="H124" s="34" t="n">
         <v>45974</v>
       </c>
       <c r="I124" s="4" t="inlineStr">
@@ -5908,10 +5929,10 @@
           <t>Монтаж устройства внутриквартирного пожаротушения систем В1.1 с отм. +4.650 до отм +46.650, со 2 по 16 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G125" s="27" t="n">
+      <c r="G125" s="34" t="n">
         <v>45952</v>
       </c>
-      <c r="H125" s="27" t="n">
+      <c r="H125" s="34" t="n">
         <v>45967</v>
       </c>
       <c r="I125" s="4" t="inlineStr">
@@ -5952,10 +5973,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов систем В1.1,Т3.1,Т4.1 и В1 от узла ввода до насосной (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G126" s="27" t="n">
+      <c r="G126" s="34" t="n">
         <v>45952</v>
       </c>
-      <c r="H126" s="27" t="n">
+      <c r="H126" s="34" t="n">
         <v>45967</v>
       </c>
       <c r="I126" s="4" t="inlineStr">
@@ -5992,8 +6013,8 @@
         </is>
       </c>
       <c r="F127" s="7" t="n"/>
-      <c r="G127" s="28" t="n"/>
-      <c r="H127" s="28" t="n"/>
+      <c r="G127" s="35" t="n"/>
+      <c r="H127" s="35" t="n"/>
       <c r="I127" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -6032,10 +6053,10 @@
           <t>Изоляция полипропиленовых и стальных трубопроводов систем В1.1,Т3.1,Т4.1 и В1 от узла ввода до насосной с отм. -1.250 до отм. +48.150, с подвала по 16 этаж в/о 1с-10с/Ас-Ис (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G128" s="27" t="n">
+      <c r="G128" s="34" t="n">
         <v>45866</v>
       </c>
-      <c r="H128" s="27" t="n">
+      <c r="H128" s="34" t="n">
         <v>45869</v>
       </c>
       <c r="I128" s="4" t="inlineStr">
@@ -6076,10 +6097,10 @@
           <t>Проведение промывки трубопроводов системы ХВС (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G129" s="27" t="n">
+      <c r="G129" s="34" t="n">
         <v>45870</v>
       </c>
-      <c r="H129" s="27" t="n">
+      <c r="H129" s="34" t="n">
         <v>45874</v>
       </c>
       <c r="I129" s="4" t="inlineStr">
@@ -6116,8 +6137,8 @@
         </is>
       </c>
       <c r="F130" s="9" t="n"/>
-      <c r="G130" s="29" t="n"/>
-      <c r="H130" s="29" t="n"/>
+      <c r="G130" s="36" t="n"/>
+      <c r="H130" s="36" t="n"/>
       <c r="I130" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -6152,8 +6173,8 @@
         </is>
       </c>
       <c r="F131" s="9" t="n"/>
-      <c r="G131" s="29" t="n"/>
-      <c r="H131" s="29" t="n"/>
+      <c r="G131" s="36" t="n"/>
+      <c r="H131" s="36" t="n"/>
       <c r="I131" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -6188,8 +6209,8 @@
         </is>
       </c>
       <c r="F132" s="9" t="n"/>
-      <c r="G132" s="29" t="n"/>
-      <c r="H132" s="29" t="n"/>
+      <c r="G132" s="36" t="n"/>
+      <c r="H132" s="36" t="n"/>
       <c r="I132" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -6224,8 +6245,8 @@
         </is>
       </c>
       <c r="F133" s="9" t="n"/>
-      <c r="G133" s="29" t="n"/>
-      <c r="H133" s="29" t="n"/>
+      <c r="G133" s="36" t="n"/>
+      <c r="H133" s="36" t="n"/>
       <c r="I133" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -6260,8 +6281,8 @@
         </is>
       </c>
       <c r="F134" s="9" t="n"/>
-      <c r="G134" s="29" t="n"/>
-      <c r="H134" s="29" t="n"/>
+      <c r="G134" s="36" t="n"/>
+      <c r="H134" s="36" t="n"/>
       <c r="I134" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -6304,10 +6325,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +52.650, 18 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G135" s="27" t="n">
+      <c r="G135" s="34" t="n">
         <v>45643</v>
       </c>
-      <c r="H135" s="27" t="n">
+      <c r="H135" s="34" t="n">
         <v>45645</v>
       </c>
       <c r="I135" s="4" t="inlineStr">
@@ -6348,10 +6369,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +55.650, 19 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G136" s="27" t="n">
+      <c r="G136" s="34" t="n">
         <v>45646</v>
       </c>
-      <c r="H136" s="27" t="n">
+      <c r="H136" s="34" t="n">
         <v>45647</v>
       </c>
       <c r="I136" s="4" t="inlineStr">
@@ -6392,10 +6413,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +58.650, 20 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G137" s="27" t="n">
+      <c r="G137" s="34" t="n">
         <v>45648</v>
       </c>
-      <c r="H137" s="27" t="n">
+      <c r="H137" s="34" t="n">
         <v>45649</v>
       </c>
       <c r="I137" s="4" t="inlineStr">
@@ -6436,10 +6457,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +61.650, 21 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G138" s="27" t="n">
+      <c r="G138" s="34" t="n">
         <v>45650</v>
       </c>
-      <c r="H138" s="27" t="n">
+      <c r="H138" s="34" t="n">
         <v>45651</v>
       </c>
       <c r="I138" s="4" t="inlineStr">
@@ -6480,10 +6501,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +64.650, 22 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G139" s="27" t="n">
+      <c r="G139" s="34" t="n">
         <v>45652</v>
       </c>
-      <c r="H139" s="27" t="n">
+      <c r="H139" s="34" t="n">
         <v>45654</v>
       </c>
       <c r="I139" s="4" t="inlineStr">
@@ -6524,10 +6545,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +67.650, 23 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G140" s="27" t="n">
+      <c r="G140" s="34" t="n">
         <v>45655</v>
       </c>
-      <c r="H140" s="27" t="n">
+      <c r="H140" s="34" t="n">
         <v>45657</v>
       </c>
       <c r="I140" s="4" t="inlineStr">
@@ -6568,10 +6589,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +70.650, 24 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G141" s="27" t="n">
+      <c r="G141" s="34" t="n">
         <v>45658</v>
       </c>
-      <c r="H141" s="27" t="n">
+      <c r="H141" s="34" t="n">
         <v>45660</v>
       </c>
       <c r="I141" s="4" t="inlineStr">
@@ -6612,10 +6633,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +73.650, 25 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G142" s="27" t="n">
+      <c r="G142" s="34" t="n">
         <v>45672</v>
       </c>
-      <c r="H142" s="27" t="n">
+      <c r="H142" s="34" t="n">
         <v>45674</v>
       </c>
       <c r="I142" s="4" t="inlineStr">
@@ -6656,10 +6677,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +76.650, 26 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G143" s="27" t="n">
+      <c r="G143" s="34" t="n">
         <v>45675</v>
       </c>
-      <c r="H143" s="27" t="n">
+      <c r="H143" s="34" t="n">
         <v>45677</v>
       </c>
       <c r="I143" s="4" t="inlineStr">
@@ -6700,10 +6721,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +79.650, 27 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G144" s="27" t="n">
+      <c r="G144" s="34" t="n">
         <v>45678</v>
       </c>
-      <c r="H144" s="27" t="n">
+      <c r="H144" s="34" t="n">
         <v>45680</v>
       </c>
       <c r="I144" s="4" t="inlineStr">
@@ -6744,10 +6765,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +82.650, 28 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G145" s="27" t="n">
+      <c r="G145" s="34" t="n">
         <v>45681</v>
       </c>
-      <c r="H145" s="27" t="n">
+      <c r="H145" s="34" t="n">
         <v>45683</v>
       </c>
       <c r="I145" s="4" t="inlineStr">
@@ -6788,10 +6809,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +85.650, 29 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G146" s="27" t="n">
+      <c r="G146" s="34" t="n">
         <v>45684</v>
       </c>
-      <c r="H146" s="27" t="n">
+      <c r="H146" s="34" t="n">
         <v>45686</v>
       </c>
       <c r="I146" s="4" t="inlineStr">
@@ -6832,10 +6853,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +88.650, 30 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G147" s="27" t="n">
+      <c r="G147" s="34" t="n">
         <v>45687</v>
       </c>
-      <c r="H147" s="27" t="n">
+      <c r="H147" s="34" t="n">
         <v>45689</v>
       </c>
       <c r="I147" s="4" t="inlineStr">
@@ -6876,10 +6897,10 @@
           <t>Монтаж горизонтальной разводки трубопроводов из сшитого полиэтилена систем В1.2, Т3.2 на отм. +91.650, 31 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G148" s="27" t="n">
+      <c r="G148" s="34" t="n">
         <v>45690</v>
       </c>
-      <c r="H148" s="27" t="n">
+      <c r="H148" s="34" t="n">
         <v>45692</v>
       </c>
       <c r="I148" s="4" t="inlineStr">
@@ -6920,10 +6941,10 @@
           <t>Монтаж полипропиленовых трубопроводов, гильз для стояков, горизонтальных трубопроводов, неподвижных опор и запорной арматуры систем В1.2,Т3.2,Т4.2 с отм. -0.947 до отм. +93.150, с подвала по 31 этаж в/о 1с-9с/Вс-Дс (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G149" s="27" t="n">
+      <c r="G149" s="34" t="n">
         <v>45694</v>
       </c>
-      <c r="H149" s="27" t="n">
+      <c r="H149" s="34" t="n">
         <v>45696</v>
       </c>
       <c r="I149" s="4" t="inlineStr">
@@ -6964,10 +6985,10 @@
           <t>Монтаж этажных распределительных коллекторов систем В1.2, Т3.2 с отм. +49.650 до отм +91.650, с 17 по 31 этаж в/о 8с-9с/Вс-Гс (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G150" s="27" t="n">
+      <c r="G150" s="34" t="n">
         <v>45677</v>
       </c>
-      <c r="H150" s="27" t="n">
+      <c r="H150" s="34" t="n">
         <v>45952</v>
       </c>
       <c r="I150" s="4" t="inlineStr">
@@ -7008,10 +7029,10 @@
           <t>Монтаж трубопроводов и запорной арматуры к сантехническому оборудованию систем В1.2, Т3.2 с отм. +49.650 до отм +91.650, с 17 по 31 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G151" s="27" t="n">
+      <c r="G151" s="34" t="n">
         <v>45981</v>
       </c>
-      <c r="H151" s="27" t="n">
+      <c r="H151" s="34" t="n">
         <v>45983</v>
       </c>
       <c r="I151" s="4" t="inlineStr">
@@ -7052,10 +7073,10 @@
           <t>Монтаж гибких подводок и смесителей систем В1.2, Т3.2 с отм. +49.650 до отм +91.650, с 17 по 31 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G152" s="27" t="n">
+      <c r="G152" s="34" t="n">
         <v>45852</v>
       </c>
-      <c r="H152" s="27" t="n">
+      <c r="H152" s="34" t="n">
         <v>45889</v>
       </c>
       <c r="I152" s="4" t="inlineStr">
@@ -7096,10 +7117,10 @@
           <t>Монтаж устройства внутриквартирного пожаротушения систем В1.1 с отм. +49.650 до отм +91.650, с 17 по 31 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G153" s="27" t="n">
+      <c r="G153" s="34" t="n">
         <v>45968</v>
       </c>
-      <c r="H153" s="27" t="n">
+      <c r="H153" s="34" t="n">
         <v>45978</v>
       </c>
       <c r="I153" s="4" t="inlineStr">
@@ -7140,10 +7161,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов систем В1.2,Т3.2,Т4.2 (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G154" s="27" t="n">
+      <c r="G154" s="34" t="n">
         <v>45968</v>
       </c>
-      <c r="H154" s="27" t="n">
+      <c r="H154" s="34" t="n">
         <v>45978</v>
       </c>
       <c r="I154" s="4" t="inlineStr">
@@ -7180,8 +7201,8 @@
         </is>
       </c>
       <c r="F155" s="7" t="n"/>
-      <c r="G155" s="28" t="n"/>
-      <c r="H155" s="28" t="n"/>
+      <c r="G155" s="35" t="n"/>
+      <c r="H155" s="35" t="n"/>
       <c r="I155" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -7220,10 +7241,10 @@
           <t>Изоляция полипропиленовых трубопроводов систем В1.2,Т3.2,Т4.2 с отм. -0.947 до отм. +93.150,с подвала по 31 этаж в/о 1с-9с/Вс-Дс (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G156" s="27" t="n">
+      <c r="G156" s="34" t="n">
         <v>45953</v>
       </c>
-      <c r="H156" s="27" t="n">
+      <c r="H156" s="34" t="n">
         <v>45956</v>
       </c>
       <c r="I156" s="4" t="inlineStr">
@@ -7264,10 +7285,10 @@
           <t>Проведение промывки трубопроводов системы ХВС (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G157" s="27" t="n">
+      <c r="G157" s="34" t="n">
         <v>45957</v>
       </c>
-      <c r="H157" s="27" t="n">
+      <c r="H157" s="34" t="n">
         <v>45961</v>
       </c>
       <c r="I157" s="4" t="inlineStr">
@@ -7304,8 +7325,8 @@
         </is>
       </c>
       <c r="F158" s="9" t="n"/>
-      <c r="G158" s="29" t="n"/>
-      <c r="H158" s="29" t="n"/>
+      <c r="G158" s="36" t="n"/>
+      <c r="H158" s="36" t="n"/>
       <c r="I158" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7340,8 +7361,8 @@
         </is>
       </c>
       <c r="F159" s="9" t="n"/>
-      <c r="G159" s="29" t="n"/>
-      <c r="H159" s="29" t="n"/>
+      <c r="G159" s="36" t="n"/>
+      <c r="H159" s="36" t="n"/>
       <c r="I159" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7376,8 +7397,8 @@
         </is>
       </c>
       <c r="F160" s="9" t="n"/>
-      <c r="G160" s="29" t="n"/>
-      <c r="H160" s="29" t="n"/>
+      <c r="G160" s="36" t="n"/>
+      <c r="H160" s="36" t="n"/>
       <c r="I160" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7412,8 +7433,8 @@
         </is>
       </c>
       <c r="F161" s="9" t="n"/>
-      <c r="G161" s="29" t="n"/>
-      <c r="H161" s="29" t="n"/>
+      <c r="G161" s="36" t="n"/>
+      <c r="H161" s="36" t="n"/>
       <c r="I161" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7448,8 +7469,8 @@
         </is>
       </c>
       <c r="F162" s="9" t="n"/>
-      <c r="G162" s="29" t="n"/>
-      <c r="H162" s="29" t="n"/>
+      <c r="G162" s="36" t="n"/>
+      <c r="H162" s="36" t="n"/>
       <c r="I162" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7492,10 +7513,10 @@
           <t>Монтаж трубопроводов к сантехническому оборудованию системы бытовой канализации К1 с отм. +4.650 до отм. +91.650 в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G163" s="27" t="n">
+      <c r="G163" s="34" t="n">
         <v>45516</v>
       </c>
-      <c r="H163" s="27" t="n">
+      <c r="H163" s="34" t="n">
         <v>45748</v>
       </c>
       <c r="I163" s="4" t="inlineStr">
@@ -7536,10 +7557,10 @@
           <t>Монтаж сантехнического оборудования системы бытовой канализации К1 с отм. +4.650 до отм. +91.650, со 2 по 31 этаж в/о 1с-11с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G164" s="27" t="n">
+      <c r="G164" s="34" t="n">
         <v>45852</v>
       </c>
-      <c r="H164" s="27" t="n">
+      <c r="H164" s="34" t="n">
         <v>45906</v>
       </c>
       <c r="I164" s="4" t="inlineStr">
@@ -7580,10 +7601,10 @@
           <t>Проведение испытания систем канализации и водостоков системы бытовой канализации К1 (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G165" s="27" t="n">
+      <c r="G165" s="34" t="n">
         <v>45952</v>
       </c>
-      <c r="H165" s="27" t="n">
+      <c r="H165" s="34" t="n">
         <v>45967</v>
       </c>
       <c r="I165" s="4" t="inlineStr">
@@ -7620,8 +7641,8 @@
         </is>
       </c>
       <c r="F166" s="11" t="n"/>
-      <c r="G166" s="30" t="n"/>
-      <c r="H166" s="30" t="n"/>
+      <c r="G166" s="37" t="n"/>
+      <c r="H166" s="37" t="n"/>
       <c r="I166" s="10" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7656,8 +7677,8 @@
         </is>
       </c>
       <c r="F167" s="9" t="n"/>
-      <c r="G167" s="29" t="n"/>
-      <c r="H167" s="29" t="n"/>
+      <c r="G167" s="36" t="n"/>
+      <c r="H167" s="36" t="n"/>
       <c r="I167" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7700,10 +7721,10 @@
           <t>Монтаж трубопроводов к сантехническому оборудованию системы бытовой канализации встроенных помещений К1.1 на отм. -0.210, 1 этаж в/о 2с-8с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G168" s="27" t="n">
+      <c r="G168" s="34" t="n">
         <v>45985</v>
       </c>
-      <c r="H168" s="27" t="n">
+      <c r="H168" s="34" t="n">
         <v>45986</v>
       </c>
       <c r="I168" s="4" t="inlineStr">
@@ -7748,10 +7769,10 @@
           <t>Монтаж сантехнического оборудования системы бытовой канализации встроенных помещений К1.1 на отм. -0.210, 1 этаж в/о 2с-8с/Бс-Ес (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G169" s="27" t="n">
+      <c r="G169" s="34" t="n">
         <v>45987</v>
       </c>
-      <c r="H169" s="27" t="n">
+      <c r="H169" s="34" t="n">
         <v>45987</v>
       </c>
       <c r="I169" s="4" t="inlineStr">
@@ -7796,10 +7817,10 @@
           <t>Проведение испытания систем канализации и водостоков системы бытовой канализации встроенных помещений К1.1 (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G170" s="27" t="n">
+      <c r="G170" s="34" t="n">
         <v>45988</v>
       </c>
-      <c r="H170" s="27" t="n">
+      <c r="H170" s="34" t="n">
         <v>45988</v>
       </c>
       <c r="I170" s="4" t="inlineStr">
@@ -7840,8 +7861,8 @@
         </is>
       </c>
       <c r="F171" s="11" t="n"/>
-      <c r="G171" s="30" t="n"/>
-      <c r="H171" s="30" t="n"/>
+      <c r="G171" s="37" t="n"/>
+      <c r="H171" s="37" t="n"/>
       <c r="I171" s="10" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7876,8 +7897,8 @@
         </is>
       </c>
       <c r="F172" s="9" t="n"/>
-      <c r="G172" s="29" t="n"/>
-      <c r="H172" s="29" t="n"/>
+      <c r="G172" s="36" t="n"/>
+      <c r="H172" s="36" t="n"/>
       <c r="I172" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -7921,10 +7942,10 @@
           <t>Проведение испытания систем канализации и водостоков системы внутреннего водостока К2 (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G173" s="27" t="n">
+      <c r="G173" s="34" t="n">
         <v>45524</v>
       </c>
-      <c r="H173" s="27" t="n">
+      <c r="H173" s="34" t="n">
         <v>45737</v>
       </c>
       <c r="I173" s="4" t="inlineStr">
@@ -7961,8 +7982,8 @@
         </is>
       </c>
       <c r="F174" s="11" t="n"/>
-      <c r="G174" s="30" t="n"/>
-      <c r="H174" s="30" t="n"/>
+      <c r="G174" s="37" t="n"/>
+      <c r="H174" s="37" t="n"/>
       <c r="I174" s="10" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -8001,10 +8022,10 @@
           <t>Освидетельствование участков сетей инженерно-технического обеспечения системы внутреннего водостока К2 (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G175" s="27" t="n">
+      <c r="G175" s="34" t="n">
         <v>45911</v>
       </c>
-      <c r="H175" s="27" t="n">
+      <c r="H175" s="34" t="n">
         <v>45913</v>
       </c>
       <c r="I175" s="4" t="inlineStr">
@@ -8041,8 +8062,8 @@
         </is>
       </c>
       <c r="F176" s="9" t="n"/>
-      <c r="G176" s="29" t="n"/>
-      <c r="H176" s="29" t="n"/>
+      <c r="G176" s="36" t="n"/>
+      <c r="H176" s="36" t="n"/>
       <c r="I176" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -8085,10 +8106,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов системы напорной дренажной канализации К13, К13н, К14н (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G177" s="27" t="n">
+      <c r="G177" s="34" t="n">
         <v>45531</v>
       </c>
-      <c r="H177" s="27" t="n">
+      <c r="H177" s="34" t="n">
         <v>45910</v>
       </c>
       <c r="I177" s="4" t="inlineStr">
@@ -8125,8 +8146,8 @@
         </is>
       </c>
       <c r="F178" s="7" t="n"/>
-      <c r="G178" s="28" t="n"/>
-      <c r="H178" s="28" t="n"/>
+      <c r="G178" s="35" t="n"/>
+      <c r="H178" s="35" t="n"/>
       <c r="I178" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -8165,10 +8186,10 @@
           <t>Проведение испытания систем канализации и водостоков системы напорной дренажной канализации К13, К13н, К14н (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G179" s="27" t="n">
+      <c r="G179" s="34" t="n">
         <v>45911</v>
       </c>
-      <c r="H179" s="27" t="n">
+      <c r="H179" s="34" t="n">
         <v>45911</v>
       </c>
       <c r="I179" s="4" t="inlineStr">
@@ -8205,8 +8226,8 @@
         </is>
       </c>
       <c r="F180" s="11" t="n"/>
-      <c r="G180" s="30" t="n"/>
-      <c r="H180" s="30" t="n"/>
+      <c r="G180" s="37" t="n"/>
+      <c r="H180" s="37" t="n"/>
       <c r="I180" s="10" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -8241,8 +8262,8 @@
         </is>
       </c>
       <c r="F181" s="13" t="n"/>
-      <c r="G181" s="31" t="n"/>
-      <c r="H181" s="31" t="n"/>
+      <c r="G181" s="38" t="n"/>
+      <c r="H181" s="38" t="n"/>
       <c r="I181" s="12" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -8277,8 +8298,8 @@
         </is>
       </c>
       <c r="F182" s="9" t="n"/>
-      <c r="G182" s="29" t="n"/>
-      <c r="H182" s="29" t="n"/>
+      <c r="G182" s="36" t="n"/>
+      <c r="H182" s="36" t="n"/>
       <c r="I182" s="8" t="inlineStr">
         <is>
           <t>08.12.2025</t>
@@ -8322,10 +8343,10 @@
           <t>Монтаж пожарного оборудования системы противопожарного водопровода В2.1 с отм. -3.350 до отм. +49.150, с подвала по 16 этаж в/о 1с-11с/Бс-Ис (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G183" s="27" t="n">
+      <c r="G183" s="34" t="n">
         <v>45526</v>
       </c>
-      <c r="H183" s="27" t="n">
+      <c r="H183" s="34" t="n">
         <v>45917</v>
       </c>
       <c r="I183" s="4" t="inlineStr">
@@ -8366,10 +8387,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов системы противопожарного водопровода В2.1 (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G184" s="27" t="n">
+      <c r="G184" s="34" t="n">
         <v>45526</v>
       </c>
-      <c r="H184" s="27" t="n">
+      <c r="H184" s="34" t="n">
         <v>45917</v>
       </c>
       <c r="I184" s="4" t="inlineStr">
@@ -8406,8 +8427,8 @@
         </is>
       </c>
       <c r="F185" s="7" t="n"/>
-      <c r="G185" s="28" t="n"/>
-      <c r="H185" s="28" t="n"/>
+      <c r="G185" s="35" t="n"/>
+      <c r="H185" s="35" t="n"/>
       <c r="I185" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -8446,10 +8467,10 @@
           <t>Зачеканка гильз в местах прохода трубопроводов через ограждающие конструкции систем противопожарного водопровода В2.1 с отм. -2.050 до отм. +46.650, с подвала по 16 этаж в/о 1с-11с/Бс-Ис (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G186" s="27" t="n">
+      <c r="G186" s="34" t="n">
         <v>45918</v>
       </c>
-      <c r="H186" s="27" t="n">
+      <c r="H186" s="34" t="n">
         <v>45919</v>
       </c>
       <c r="I186" s="4" t="inlineStr">
@@ -8494,10 +8515,10 @@
           <t>Испытание на водоотдачу внутреннего противопожарного водопровода (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G187" s="27" t="n">
+      <c r="G187" s="34" t="n">
         <v>45920</v>
       </c>
-      <c r="H187" s="27" t="n">
+      <c r="H187" s="34" t="n">
         <v>45921</v>
       </c>
       <c r="I187" s="4" t="inlineStr">
@@ -8534,8 +8555,8 @@
         </is>
       </c>
       <c r="F188" s="9" t="n"/>
-      <c r="G188" s="29" t="n"/>
-      <c r="H188" s="29" t="n"/>
+      <c r="G188" s="36" t="n"/>
+      <c r="H188" s="36" t="n"/>
       <c r="I188" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -8570,8 +8591,8 @@
         </is>
       </c>
       <c r="F189" s="15" t="n"/>
-      <c r="G189" s="32" t="n"/>
-      <c r="H189" s="32" t="n"/>
+      <c r="G189" s="39" t="n"/>
+      <c r="H189" s="39" t="n"/>
       <c r="I189" s="14" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -8606,8 +8627,8 @@
         </is>
       </c>
       <c r="F190" s="9" t="n"/>
-      <c r="G190" s="29" t="n"/>
-      <c r="H190" s="29" t="n"/>
+      <c r="G190" s="36" t="n"/>
+      <c r="H190" s="36" t="n"/>
       <c r="I190" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -8650,10 +8671,10 @@
           <t>Монтаж пожарного оборудования системы противопожарного водопровода В2.2 с отм. +50.950 до отм. +94.630, с 17 этажа по тех. чердак в/о 1с-9с/Бс-Дс (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G191" s="27" t="n">
+      <c r="G191" s="34" t="n">
         <v>45526</v>
       </c>
-      <c r="H191" s="27" t="n">
+      <c r="H191" s="34" t="n">
         <v>45876</v>
       </c>
       <c r="I191" s="4" t="inlineStr">
@@ -8694,10 +8715,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов системы противопожарного водопровода В2.2 (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G192" s="27" t="n">
+      <c r="G192" s="34" t="n">
         <v>45526</v>
       </c>
-      <c r="H192" s="27" t="n">
+      <c r="H192" s="34" t="n">
         <v>45876</v>
       </c>
       <c r="I192" s="4" t="inlineStr">
@@ -8734,8 +8755,8 @@
         </is>
       </c>
       <c r="F193" s="7" t="n"/>
-      <c r="G193" s="28" t="n"/>
-      <c r="H193" s="28" t="n"/>
+      <c r="G193" s="35" t="n"/>
+      <c r="H193" s="35" t="n"/>
       <c r="I193" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -8774,10 +8795,10 @@
           <t>Зачеканка гильз в местах прохода трубопроводов через ограждающие конструкции систем противопожарного водопровода В2.2 с отм. -1.071 до отм. +94.930, с подвала по тех. чердак в/о 1с-9с/Бс-Дс (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G194" s="27" t="n">
+      <c r="G194" s="34" t="n">
         <v>45877</v>
       </c>
-      <c r="H194" s="27" t="n">
+      <c r="H194" s="34" t="n">
         <v>45878</v>
       </c>
       <c r="I194" s="4" t="inlineStr">
@@ -8822,10 +8843,10 @@
           <t>Испытание на водоотдачу внутреннего противопожарного водопровода (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G195" s="27" t="n">
+      <c r="G195" s="34" t="n">
         <v>45879</v>
       </c>
-      <c r="H195" s="27" t="n">
+      <c r="H195" s="34" t="n">
         <v>45880</v>
       </c>
       <c r="I195" s="4" t="inlineStr">
@@ -8862,8 +8883,8 @@
         </is>
       </c>
       <c r="F196" s="9" t="n"/>
-      <c r="G196" s="29" t="n"/>
-      <c r="H196" s="29" t="n"/>
+      <c r="G196" s="36" t="n"/>
+      <c r="H196" s="36" t="n"/>
       <c r="I196" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -8898,8 +8919,8 @@
         </is>
       </c>
       <c r="F197" s="15" t="n"/>
-      <c r="G197" s="32" t="n"/>
-      <c r="H197" s="32" t="n"/>
+      <c r="G197" s="39" t="n"/>
+      <c r="H197" s="39" t="n"/>
       <c r="I197" s="14" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -8934,8 +8955,8 @@
         </is>
       </c>
       <c r="F198" s="9" t="n"/>
-      <c r="G198" s="29" t="n"/>
-      <c r="H198" s="29" t="n"/>
+      <c r="G198" s="36" t="n"/>
+      <c r="H198" s="36" t="n"/>
       <c r="I198" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -8978,10 +8999,10 @@
           <t>Монтаж пожарного оборудования системы автоматического пожаротушения кладовых В2 с отм. -0.887 до отм. -0.661, подвал в/о 1с-10с/Ас-Ис (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G199" s="27" t="n">
+      <c r="G199" s="34" t="n">
         <v>45981</v>
       </c>
-      <c r="H199" s="27" t="n">
+      <c r="H199" s="34" t="n">
         <v>45983</v>
       </c>
       <c r="I199" s="4" t="inlineStr">
@@ -9022,10 +9043,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов системы автоматического пожаротушения кладовых В2 (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G200" s="27" t="n">
+      <c r="G200" s="34" t="n">
         <v>45989</v>
       </c>
-      <c r="H200" s="27" t="n">
+      <c r="H200" s="34" t="n">
         <v>45989</v>
       </c>
       <c r="I200" s="4" t="inlineStr">
@@ -9062,8 +9083,8 @@
         </is>
       </c>
       <c r="F201" s="7" t="n"/>
-      <c r="G201" s="28" t="n"/>
-      <c r="H201" s="28" t="n"/>
+      <c r="G201" s="35" t="n"/>
+      <c r="H201" s="35" t="n"/>
       <c r="I201" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -9102,10 +9123,10 @@
           <t>Зачеканка гильз в местах прохода через ограждающие конструкции трубопроводов систем автоматического пожаротушения кладовых В2 с отм. -0.887 до отм. -0.210, с подвала по 1 этаж в/о 1с-10с/Ас-Ис (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G202" s="27" t="n">
+      <c r="G202" s="34" t="n">
         <v>45996</v>
       </c>
-      <c r="H202" s="27" t="n">
+      <c r="H202" s="34" t="n">
         <v>45996</v>
       </c>
       <c r="I202" s="4" t="inlineStr">
@@ -9150,10 +9171,10 @@
           <t>Испытание на водоотдачу внутреннего противопожарного водопровода (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G203" s="27" t="n">
+      <c r="G203" s="34" t="n">
         <v>45999</v>
       </c>
-      <c r="H203" s="27" t="n">
+      <c r="H203" s="34" t="n">
         <v>45999</v>
       </c>
       <c r="I203" s="4" t="inlineStr">
@@ -9190,8 +9211,8 @@
         </is>
       </c>
       <c r="F204" s="9" t="n"/>
-      <c r="G204" s="29" t="n"/>
-      <c r="H204" s="29" t="n"/>
+      <c r="G204" s="36" t="n"/>
+      <c r="H204" s="36" t="n"/>
       <c r="I204" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9230,8 +9251,8 @@
         </is>
       </c>
       <c r="F205" s="17" t="n"/>
-      <c r="G205" s="33" t="n"/>
-      <c r="H205" s="33" t="n"/>
+      <c r="G205" s="40" t="n"/>
+      <c r="H205" s="40" t="n"/>
       <c r="I205" s="16" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9270,8 +9291,8 @@
         </is>
       </c>
       <c r="F206" s="15" t="n"/>
-      <c r="G206" s="32" t="n"/>
-      <c r="H206" s="32" t="n"/>
+      <c r="G206" s="39" t="n"/>
+      <c r="H206" s="39" t="n"/>
       <c r="I206" s="14" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9306,8 +9327,8 @@
         </is>
       </c>
       <c r="F207" s="9" t="n"/>
-      <c r="G207" s="29" t="n"/>
-      <c r="H207" s="29" t="n"/>
+      <c r="G207" s="36" t="n"/>
+      <c r="H207" s="36" t="n"/>
       <c r="I207" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9350,10 +9371,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов хоз. питьевой насосной станции (сети В1, В1.1, В1.2) (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G208" s="27" t="n">
+      <c r="G208" s="34" t="n">
         <v>45763</v>
       </c>
-      <c r="H208" s="27" t="n">
+      <c r="H208" s="34" t="n">
         <v>45833</v>
       </c>
       <c r="I208" s="4" t="inlineStr">
@@ -9390,8 +9411,8 @@
         </is>
       </c>
       <c r="F209" s="7" t="n"/>
-      <c r="G209" s="28" t="n"/>
-      <c r="H209" s="28" t="n"/>
+      <c r="G209" s="35" t="n"/>
+      <c r="H209" s="35" t="n"/>
       <c r="I209" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -9430,10 +9451,10 @@
           <t>Проведение индивидуального испытания оборудования насосной станции хоз. питьевой водоснабжения (сети В1, В1.1, В1.2) (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G210" s="27" t="n">
+      <c r="G210" s="34" t="n">
         <v>45834</v>
       </c>
-      <c r="H210" s="27" t="n">
+      <c r="H210" s="34" t="n">
         <v>45836</v>
       </c>
       <c r="I210" s="4" t="inlineStr">
@@ -9470,8 +9491,8 @@
         </is>
       </c>
       <c r="F211" s="13" t="n"/>
-      <c r="G211" s="31" t="n"/>
-      <c r="H211" s="31" t="n"/>
+      <c r="G211" s="38" t="n"/>
+      <c r="H211" s="38" t="n"/>
       <c r="I211" s="12" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9506,8 +9527,8 @@
         </is>
       </c>
       <c r="F212" s="9" t="n"/>
-      <c r="G212" s="29" t="n"/>
-      <c r="H212" s="29" t="n"/>
+      <c r="G212" s="36" t="n"/>
+      <c r="H212" s="36" t="n"/>
       <c r="I212" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9542,8 +9563,8 @@
         </is>
       </c>
       <c r="F213" s="9" t="n"/>
-      <c r="G213" s="29" t="n"/>
-      <c r="H213" s="29" t="n"/>
+      <c r="G213" s="36" t="n"/>
+      <c r="H213" s="36" t="n"/>
       <c r="I213" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9578,8 +9599,8 @@
         </is>
       </c>
       <c r="F214" s="9" t="n"/>
-      <c r="G214" s="29" t="n"/>
-      <c r="H214" s="29" t="n"/>
+      <c r="G214" s="36" t="n"/>
+      <c r="H214" s="36" t="n"/>
       <c r="I214" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9622,10 +9643,10 @@
           <t>Гидростатическое испытание на герметичность трубопроводов насосной станции пожаротушения (сети В2.1, В2.2, В21) (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G215" s="27" t="n">
+      <c r="G215" s="34" t="n">
         <v>45763</v>
       </c>
-      <c r="H215" s="27" t="n">
+      <c r="H215" s="34" t="n">
         <v>45833</v>
       </c>
       <c r="I215" s="4" t="inlineStr">
@@ -9662,8 +9683,8 @@
         </is>
       </c>
       <c r="F216" s="7" t="n"/>
-      <c r="G216" s="28" t="n"/>
-      <c r="H216" s="28" t="n"/>
+      <c r="G216" s="35" t="n"/>
+      <c r="H216" s="35" t="n"/>
       <c r="I216" s="6" t="inlineStr">
         <is>
           <t>04.12.2025</t>
@@ -9702,10 +9723,10 @@
           <t>Проведение индивидуального испытания оборудования насосной станции пожаротушения (сети В2.1, В2.2, В21) (Секция №12.2)</t>
         </is>
       </c>
-      <c r="G217" s="27" t="n">
+      <c r="G217" s="34" t="n">
         <v>45834</v>
       </c>
-      <c r="H217" s="27" t="n">
+      <c r="H217" s="34" t="n">
         <v>45836</v>
       </c>
       <c r="I217" s="4" t="inlineStr">
@@ -9742,8 +9763,8 @@
         </is>
       </c>
       <c r="F218" s="13" t="n"/>
-      <c r="G218" s="31" t="n"/>
-      <c r="H218" s="31" t="n"/>
+      <c r="G218" s="38" t="n"/>
+      <c r="H218" s="38" t="n"/>
       <c r="I218" s="12" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9778,8 +9799,8 @@
         </is>
       </c>
       <c r="F219" s="15" t="n"/>
-      <c r="G219" s="32" t="n"/>
-      <c r="H219" s="32" t="n"/>
+      <c r="G219" s="39" t="n"/>
+      <c r="H219" s="39" t="n"/>
       <c r="I219" s="14" t="inlineStr">
         <is>
           <t>09.12.2025</t>
@@ -9814,8 +9835,8 @@
         </is>
       </c>
       <c r="F220" s="9" t="n"/>
-      <c r="G220" s="29" t="n"/>
-      <c r="H220" s="29" t="n"/>
+      <c r="G220" s="36" t="n"/>
+      <c r="H220" s="36" t="n"/>
       <c r="I220" s="8" t="inlineStr">
         <is>
           <t>09.12.2025</t>

</xml_diff>